<commit_message>
Matriz nueva: orden de subcategorías por número; clientes 20 y 21 con Visita Médica, Visita Médica Comercial o ambas (lista unida)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +78,42 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006B4F"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006B4F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006B4F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF006B4F"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00006B4F"/>
       <sz val="14"/>
@@ -105,7 +141,7 @@
       <color rgb="00006B4F"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +175,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF006B4F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF7D6"/>
       </patternFill>
     </fill>
@@ -148,7 +194,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -173,6 +219,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFE5D9A8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5D9A8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5D9A8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE5D9A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="00E5D9A8"/>
       </left>
       <right style="thin">
@@ -189,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -242,6 +303,17 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -633,33 +705,33 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Matriz de Epithelium Visita</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>Actualizada el 29/09/2026 · es lo que la app tiene cargado hoy</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Hoja</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>Qué contiene</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>Visitas</t>
         </is>
@@ -671,7 +743,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>Trabajo interno</t>
         </is>
@@ -683,7 +755,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Mensual</t>
         </is>
@@ -695,7 +767,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>Tipo de visita</t>
         </is>
@@ -707,7 +779,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Reglas</t>
         </is>
@@ -733,7 +805,7 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Orden alfabético, salvo Planeación Mes y las subcategorías con orden fijo (Colocación, Desarrollo Productos, Devoluciones - PQR, Mapa del Cliente y Productos Nuevos).</t>
+          <t>Objetivos en orden alfabético (salvo Planeación Mes). Subcategorías: el número en la columna A es su orden.</t>
         </is>
       </c>
     </row>
@@ -744,6 +816,18 @@
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Clasificaciones 20 y 21: al programar se marca Visita Médica, Visita Médica Comercial o ambas (lista unida).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>No cambies los encabezados (fila 4) ni el nombre de las hojas.</t>
         </is>
@@ -908,7 +992,9 @@
       <c r="I7" s="7" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
+      <c r="A8" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Acuerdo de Pago</t>
@@ -931,7 +1017,9 @@
       <c r="I8" s="12" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
+      <c r="A9" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Cobro de Factura</t>
@@ -954,7 +1042,9 @@
       <c r="I9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
+      <c r="A10" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Conciliación de Cartera</t>
@@ -977,7 +1067,9 @@
       <c r="I10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
+      <c r="A11" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Recibo de Caja</t>
@@ -1023,7 +1115,9 @@
       <c r="I12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
+      <c r="A13" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Actividades</t>
@@ -1046,7 +1140,9 @@
       <c r="I13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
+      <c r="A14" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Portafolio</t>
@@ -1069,7 +1165,9 @@
       <c r="I14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
+      <c r="A15" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Producto Nuevo</t>
@@ -1123,7 +1221,9 @@
       <c r="I16" s="7" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
+      <c r="A17" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Presentación y Documentación</t>
@@ -1150,7 +1250,9 @@
       <c r="I17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
+      <c r="A18" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Producto Codificado</t>
@@ -1177,7 +1279,9 @@
       <c r="I18" s="12" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
+      <c r="A19" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Seguimiento a la Codificación</t>
@@ -1204,7 +1308,9 @@
       <c r="I19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
+      <c r="A20" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Solicitud de Codificación</t>
@@ -1266,7 +1372,9 @@
       <c r="I21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
+      <c r="A22" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Magistral de Pedido</t>
@@ -1297,7 +1405,9 @@
       <c r="I22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
+      <c r="A23" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Magistral Individual</t>
@@ -1328,7 +1438,9 @@
       <c r="I23" s="12" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
+      <c r="A24" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Producto Nuevo</t>
@@ -1359,7 +1471,9 @@
       <c r="I24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
+      <c r="A25" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Producto Terminado</t>
@@ -1561,7 +1675,9 @@
       <c r="I30" s="7" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
+      <c r="A31" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Devolución</t>
@@ -1588,7 +1704,9 @@
       <c r="I31" s="12" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
+      <c r="A32" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Queja</t>
@@ -1619,7 +1737,9 @@
       <c r="I32" s="12" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
+      <c r="A33" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Reacondicionamiento</t>
@@ -1646,7 +1766,9 @@
       <c r="I33" s="12" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
+      <c r="A34" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Reclamo</t>
@@ -1677,7 +1799,9 @@
       <c r="I34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n"/>
+      <c r="A35" s="11" t="n">
+        <v>5</v>
+      </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Sugerencia</t>
@@ -1751,7 +1875,9 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n"/>
+      <c r="A37" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Muestra Comercial</t>
@@ -1790,7 +1916,9 @@
       <c r="I37" s="12" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n"/>
+      <c r="A38" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Muestra Médica</t>
@@ -1829,7 +1957,9 @@
       <c r="I38" s="12" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n"/>
+      <c r="A39" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Tester</t>
@@ -1875,7 +2005,9 @@
       <c r="I40" s="7" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n"/>
+      <c r="A41" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Góndola</t>
@@ -1894,7 +2026,9 @@
       <c r="I41" s="12" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n"/>
+      <c r="A42" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Material POP</t>
@@ -1913,7 +2047,9 @@
       <c r="I42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n"/>
+      <c r="A43" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Vitrina</t>
@@ -1959,7 +2095,9 @@
       <c r="I44" s="7" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n"/>
+      <c r="A45" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
           <t>Portafolio Actual</t>
@@ -1982,7 +2120,9 @@
       <c r="I45" s="12" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n"/>
+      <c r="A46" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
           <t>Productos Foco</t>
@@ -2005,7 +2145,9 @@
       <c r="I46" s="12" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n"/>
+      <c r="A47" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Productos Nuevos</t>
@@ -2028,7 +2170,9 @@
       <c r="I47" s="12" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n"/>
+      <c r="A48" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
           <t>Productos Transición</t>
@@ -2132,7 +2276,9 @@
       <c r="I51" s="7" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n"/>
+      <c r="A52" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
           <t>Lista de Precios</t>
@@ -2159,7 +2305,9 @@
       <c r="I52" s="12" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n"/>
+      <c r="A53" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
           <t>Negociación</t>
@@ -2186,7 +2334,9 @@
       <c r="I53" s="12" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n"/>
+      <c r="A54" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
           <t>Chequeo de Precios</t>
@@ -2256,7 +2406,9 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="n"/>
+      <c r="A56" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
           <t>Codificación</t>
@@ -2287,7 +2439,9 @@
       <c r="I56" s="12" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="n"/>
+      <c r="A57" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
           <t>Entrega de Muestra</t>
@@ -2318,7 +2472,9 @@
       <c r="I57" s="12" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="n"/>
+      <c r="A58" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
           <t>Material de Apoyo</t>
@@ -2349,7 +2505,9 @@
       <c r="I58" s="12" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n"/>
+      <c r="A59" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
           <t>Presentación del Producto</t>
@@ -2419,7 +2577,9 @@
       <c r="I60" s="7" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n"/>
+      <c r="A61" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
           <t>Inscripción del Médico</t>
@@ -2442,10 +2602,12 @@
       <c r="I61" s="12" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="n"/>
+      <c r="A62" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Presentación del Protocolo</t>
+          <t>Presentación Protocolo Médico</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
@@ -2469,7 +2631,9 @@
       <c r="I62" s="12" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="n"/>
+      <c r="A63" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
           <t>Seguimiento</t>
@@ -2492,7 +2656,9 @@
       <c r="I63" s="12" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="n"/>
+      <c r="A64" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
           <t>Solicitud y Recolección de Información</t>
@@ -3902,14 +4068,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>Tipo de visita según la clasificación del cliente</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>X en los tipos de visita donde sale cada clasificación. Con X en Visita Médica y Visita Comercial (20 y 21) el vendedor marca una, otra o ambas; con las dos marcadas se usan los objetivos de "Visita Médica Comercial" (hoja Visitas).</t>
         </is>
@@ -3969,13 +4135,13 @@
           <t>Cliente (5)</t>
         </is>
       </c>
-      <c r="E5" s="27" t="n"/>
-      <c r="F5" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G5" s="27" t="n"/>
+      <c r="E5" s="34" t="n"/>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="n">
@@ -3994,13 +4160,13 @@
           <t>Cliente (27)</t>
         </is>
       </c>
-      <c r="E6" s="27" t="n"/>
-      <c r="F6" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G6" s="27" t="n"/>
+      <c r="E6" s="34" t="n"/>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="25" t="n">
@@ -4019,9 +4185,9 @@
           <t>Punto de Venta (220) · Centro de Distribucion (2)</t>
         </is>
       </c>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="inlineStr">
+      <c r="E7" s="34" t="n"/>
+      <c r="F7" s="34" t="n"/>
+      <c r="G7" s="34" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -4044,13 +4210,13 @@
           <t>Cliente (10)</t>
         </is>
       </c>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G8" s="27" t="n"/>
+      <c r="E8" s="34" t="n"/>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="25" t="n">
@@ -4069,13 +4235,13 @@
           <t>Cliente (2)</t>
         </is>
       </c>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G9" s="27" t="n"/>
+      <c r="E9" s="34" t="n"/>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="25" t="n">
@@ -4094,17 +4260,17 @@
           <t>Medico Accionista - Panel Visita Medica (19) · Accionista Epithelium (2)</t>
         </is>
       </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G10" s="34" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="25" t="n">
@@ -4123,17 +4289,17 @@
           <t>Cliente - Medico Panel (42) · Cliente (2) · Medico Panel Visita Medica (1)</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
@@ -4152,13 +4318,13 @@
           <t>Medico Panel Visita Medica (147) · Medico - Ateneo Sanitas - Centro Dermatologico Federico Lleras Acosta E.S.E (20) · Medico - Ateneo Hospital San Jose -Fundacion Universitaria de la Salud - FUCS (18) · Medico - Ateneo Universidad del Bosque (12) · Medico - Ateneo Hospital Militar Central (6) · Medico - Protocolo Medico (2) · Cliente - Medico Panel (2)</t>
         </is>
       </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n"/>
-      <c r="G12" s="27" t="n"/>
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="n"/>
+      <c r="G12" s="34" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
@@ -4177,13 +4343,13 @@
           <t>Cliente (4)</t>
         </is>
       </c>
-      <c r="E13" s="27" t="n"/>
-      <c r="F13" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="E13" s="34" t="n"/>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
@@ -4202,13 +4368,13 @@
           <t>Cliente (12)</t>
         </is>
       </c>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G14" s="27" t="n"/>
+      <c r="E14" s="34" t="n"/>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
@@ -4227,13 +4393,13 @@
           <t>Cliente (2)</t>
         </is>
       </c>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G15" s="27" t="n"/>
+      <c r="E15" s="34" t="n"/>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="n">
@@ -4252,13 +4418,13 @@
           <t>Cliente (3)</t>
         </is>
       </c>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G16" s="27" t="n"/>
+      <c r="E16" s="34" t="n"/>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
@@ -4277,13 +4443,13 @@
           <t>Cliente (1) · Entidad Gubernamental Cliente (1)</t>
         </is>
       </c>
-      <c r="E17" s="27" t="n"/>
-      <c r="F17" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G17" s="27" t="n"/>
+      <c r="E17" s="34" t="n"/>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="25" t="n">
@@ -4302,13 +4468,13 @@
           <t>Cliente (2)</t>
         </is>
       </c>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G18" s="27" t="n"/>
+      <c r="E18" s="34" t="n"/>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G18" s="34" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="25" t="n">
@@ -4327,13 +4493,13 @@
           <t>Cliente (4)</t>
         </is>
       </c>
-      <c r="E19" s="27" t="n"/>
-      <c r="F19" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G19" s="27" t="n"/>
+      <c r="E19" s="34" t="n"/>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G19" s="34" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="25" t="n">
@@ -4352,16 +4518,16 @@
           <t>Cliente (10) · Accionista Epithelium (1)</t>
         </is>
       </c>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="27" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G20" s="27" t="n"/>
+      <c r="E20" s="34" t="n"/>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Total clientes en la maestra: 579 · Amarillo fuerte = clasificación sin X (sale en todos los tipos)</t>
         </is>

</xml_diff>

<commit_message>
Matriz nueva: Visita Comercial pasa a Visita Cliente, Mapa del Cliente, trabajo interno reorganizado y tildes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -282,6 +282,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -289,19 +301,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -401,7 +401,7 @@
     <tableColumn id="3" name="Clientes"/>
     <tableColumn id="4" name="Etiquetas en la maestra"/>
     <tableColumn id="5" name="Visita Médica"/>
-    <tableColumn id="6" name="Visita Comercial"/>
+    <tableColumn id="6" name="Visita Cliente"/>
     <tableColumn id="7" name="Punto de Venta"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showRowStripes="1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Actualizada el 29/09/2026 · es lo que la app tiene cargado hoy</t>
+          <t>Actualizada el 30/09/2026 · es lo que la app tiene cargado hoy</t>
         </is>
       </c>
     </row>
@@ -736,9 +736,9 @@
           <t>Visitas</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>Objetivos (fila verde, ✓) y subcategorías (X) por tipo de visita: Visita Médica, Visita Médica Comercial (20 y 21 con las dos marcadas), Visita Comercial, Punto de Venta y Contacto nuevo.</t>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Objetivos (fila verde, ✓) y subcategorías (X) por tipo de visita: Visita Médica, Visita Médica Comercial (20 y 21 con las dos marcadas), Visita Cliente, Punto de Venta y Contacto nuevo.</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
           <t>Trabajo interno</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Objetivos y subcategorías de Oficina, Fuera de la Oficina y Planeación Mes.</t>
         </is>
@@ -760,7 +760,7 @@
           <t>Mensual</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Parrilla Promocional y Actividades de cada mes (subcategorías variables).</t>
         </is>
@@ -772,7 +772,7 @@
           <t>Tipo de visita</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>En qué tipo de visita sale cada clasificación de cliente de la Maestra.</t>
         </is>
@@ -791,7 +791,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Nombres en nombre propio (NOMPROPIO), con de/del/la/y en minúscula: "Chequeo de Precios".</t>
         </is>
@@ -803,7 +803,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>Objetivos en orden alfabético (salvo Planeación Mes). Subcategorías: el número en la columna A es su orden.</t>
         </is>
@@ -815,7 +815,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Clasificaciones 20 y 21: al programar se marca Visita Médica, Visita Médica Comercial o ambas (lista unida).</t>
         </is>
@@ -827,7 +827,7 @@
           <t>•</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>No cambies los encabezados (fila 4) ni el nombre de las hojas.</t>
         </is>
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -878,7 +878,7 @@
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Objetivo</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Visita Comercial</t>
+          <t>Visita Cliente</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Contacto nuevo · Visita Comercial</t>
+          <t>Contacto nuevo · Visita Cliente</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1018,7 +1018,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
@@ -1196,11 +1196,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n"/>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -1240,22 +1236,18 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F17" s="12" t="n"/>
       <c r="G17" s="12" t="n"/>
       <c r="H17" s="12" t="n"/>
       <c r="I17" s="12" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Producto Codificado</t>
+          <t>Seguimiento a la Codificación</t>
         </is>
       </c>
       <c r="C18" s="12" t="n"/>
@@ -1280,24 +1272,16 @@
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Seguimiento a la Codificación</t>
+          <t>Vectorización</t>
         </is>
       </c>
       <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
       <c r="F19" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1308,76 +1292,76 @@
       <c r="I19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Solicitud de Codificación</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
-      <c r="I20" s="12" t="n"/>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Colocación</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="n"/>
+      <c r="A21" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Magistral de Pedido</t>
+          <t>Magistral Individual</t>
         </is>
       </c>
       <c r="C22" s="12" t="n"/>
@@ -1406,11 +1390,11 @@
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Magistral Individual</t>
+          <t>Producto Nuevo</t>
         </is>
       </c>
       <c r="C23" s="12" t="n"/>
@@ -1439,11 +1423,11 @@
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Producto Nuevo</t>
+          <t>Producto Terminado</t>
         </is>
       </c>
       <c r="C24" s="12" t="n"/>
@@ -1471,78 +1455,84 @@
       <c r="I24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo Productos</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Producto Terminado</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I25" s="12" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo Productos</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="n"/>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Ajuste de Fórmula</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
+      <c r="A27" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Ajuste de Fórmula</t>
+          <t>Fórmula Magistral Nueva</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -1574,10 +1564,12 @@
       <c r="I27" s="12" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
+      <c r="A28" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Fórmula Magistral Nueva</t>
+          <t>Muestra de Desarrollo</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1609,81 +1601,79 @@
       <c r="I28" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Muestra de Desarrollo</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="n"/>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Devoluciones - PQR</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Devoluciones - PQR</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
+      <c r="A30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Devolución</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Devolución</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="n"/>
+          <t>Queja</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1705,18 +1695,14 @@
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Queja</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Reacondicionamiento</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n"/>
       <c r="D32" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1727,25 +1713,25 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F32" s="12" t="n"/>
       <c r="G32" s="12" t="n"/>
       <c r="H32" s="12" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Reacondicionamiento</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="n"/>
+          <t>Reclamo</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1767,11 +1753,11 @@
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Reclamo</t>
+          <t>Sugerencia</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -1799,88 +1785,96 @@
       <c r="I34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>Sugerencia</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Entrega de Muestras</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Entrega de Muestras</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A36" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Muestra Comercial</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Muestra Comercial</t>
+          <t>Muestra Médica</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
@@ -1898,11 +1892,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F37" s="12" t="n"/>
       <c r="G37" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1917,105 +1907,97 @@
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Exhibición</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Muestra Médica</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I38" s="12" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="n"/>
-      <c r="D39" s="12" t="n"/>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G39" s="12" t="n"/>
-      <c r="H39" s="12" t="n"/>
-      <c r="I39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Exhibición</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
-      <c r="I40" s="7" t="n"/>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Góndola</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40" s="12" t="n"/>
+      <c r="I40" s="12" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>Góndola</t>
+          <t>Material POP</t>
         </is>
       </c>
       <c r="C41" s="12" t="n"/>
       <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -2027,16 +2009,20 @@
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Material POP</t>
+          <t>Vitrina</t>
         </is>
       </c>
       <c r="C42" s="12" t="n"/>
       <c r="D42" s="12" t="n"/>
-      <c r="E42" s="12" t="n"/>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -2047,60 +2033,64 @@
       <c r="I42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Vitrina</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="n"/>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G43" s="12" t="n"/>
-      <c r="H43" s="12" t="n"/>
-      <c r="I43" s="12" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Mapa del Cliente</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Mapa del Cliente - Ampliación Portafolio</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="7" t="n"/>
-      <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
+      <c r="A44" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Portafolio Actual</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
+      <c r="H44" s="12" t="n"/>
+      <c r="I44" s="12" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>Portafolio Actual</t>
+          <t>Productos Foco</t>
         </is>
       </c>
       <c r="C45" s="12" t="n"/>
@@ -2121,11 +2111,11 @@
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>Productos Foco</t>
+          <t>Productos Nuevos</t>
         </is>
       </c>
       <c r="C46" s="12" t="n"/>
@@ -2146,11 +2136,11 @@
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Productos Nuevos</t>
+          <t>Productos Transición</t>
         </is>
       </c>
       <c r="C47" s="12" t="n"/>
@@ -2170,118 +2160,106 @@
       <c r="I47" s="12" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B48" s="11" t="inlineStr">
-        <is>
-          <t>Productos Transición</t>
-        </is>
-      </c>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="12" t="n"/>
-      <c r="I48" s="12" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Parrilla Promocional</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Parrilla Promocional</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H49" s="7" t="n"/>
-      <c r="I49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="n"/>
+      <c r="D49" s="10" t="n"/>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="10" t="n"/>
+      <c r="I49" s="10" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="n"/>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="n"/>
-      <c r="D50" s="10" t="n"/>
-      <c r="E50" s="10" t="n"/>
-      <c r="F50" s="10" t="n"/>
-      <c r="G50" s="10" t="n"/>
-      <c r="H50" s="10" t="n"/>
-      <c r="I50" s="10" t="n"/>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Precios</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Precios</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="n"/>
-      <c r="H51" s="7" t="n"/>
-      <c r="I51" s="7" t="n"/>
+      <c r="A51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Lista de Precios</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="12" t="n"/>
+      <c r="I51" s="12" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Lista de Precios</t>
+          <t>Negociación</t>
         </is>
       </c>
       <c r="C52" s="12" t="n"/>
@@ -2295,22 +2273,18 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F52" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F52" s="12" t="n"/>
       <c r="G52" s="12" t="n"/>
       <c r="H52" s="12" t="n"/>
       <c r="I52" s="12" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Negociación</t>
+          <t>Chequeo de Precios</t>
         </is>
       </c>
       <c r="C53" s="12" t="n"/>
@@ -2334,84 +2308,84 @@
       <c r="I53" s="12" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B54" s="11" t="inlineStr">
-        <is>
-          <t>Chequeo de Precios</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G54" s="12" t="n"/>
-      <c r="H54" s="12" t="n"/>
-      <c r="I54" s="12" t="n"/>
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Productos Nuevos</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Productos Nuevos</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A55" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>Codificación</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="12" t="n"/>
+      <c r="H55" s="12" t="n"/>
+      <c r="I55" s="12" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Codificación</t>
+          <t>Entrega de Muestra</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
@@ -2440,11 +2414,11 @@
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Entrega de Muestra</t>
+          <t>Material de Apoyo</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
@@ -2473,11 +2447,11 @@
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Material de Apoyo</t>
+          <t>Presentación del Producto</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
@@ -2500,89 +2474,81 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G58" s="12" t="n"/>
-      <c r="H58" s="12" t="n"/>
-      <c r="I58" s="12" t="n"/>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>Presentación del Producto</t>
-        </is>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Protocolo Médico</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="n"/>
+      <c r="I59" s="7" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>Protocolo Médico</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n"/>
-      <c r="F60" s="7" t="n"/>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H60" s="7" t="n"/>
-      <c r="I60" s="7" t="n"/>
+      <c r="A60" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Inscripción del Médico</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Inscripción del Médico</t>
+          <t>Presentación Protocolo Médico</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
@@ -2597,17 +2563,21 @@
       </c>
       <c r="E61" s="12" t="n"/>
       <c r="F61" s="12" t="n"/>
-      <c r="G61" s="12" t="n"/>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H61" s="12" t="n"/>
       <c r="I61" s="12" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Presentación Protocolo Médico</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
@@ -2622,21 +2592,17 @@
       </c>
       <c r="E62" s="12" t="n"/>
       <c r="F62" s="12" t="n"/>
-      <c r="G62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G62" s="12" t="n"/>
       <c r="H62" s="12" t="n"/>
       <c r="I62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Solicitud y Recolección de Información</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
@@ -2655,34 +2621,9 @@
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
-    <row r="64">
-      <c r="A64" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>Solicitud y Recolección de Información</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="12" t="n"/>
-      <c r="I64" s="12" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C5:I105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:I104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,✓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2696,7 +2637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2721,7 +2662,7 @@
     <row r="4" ht="44.1" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Objetivo</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
@@ -2761,10 +2702,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n"/>
+      <c r="A6" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Ajustes al Plan</t>
+          <t>Elaboración Visiplan Mes</t>
         </is>
       </c>
       <c r="C6" s="12" t="n"/>
@@ -2776,10 +2719,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
+      <c r="A7" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Clientes a Visitar por Día</t>
+          <t>Revisión del Cumplimiento del Mes Anterior</t>
         </is>
       </c>
       <c r="C7" s="12" t="n"/>
@@ -2791,274 +2736,338 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Frecuencia de Visita por Cliente</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Diagnóstico de Zona</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Revisión del Cumplimiento del Mes Anterior</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Plan de Acción</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Diagnóstico de Zona</t>
+          <t>Plan de Trabajo Diario</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
+      <c r="A11" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Cartera de la Zona</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Confirmación de Citas</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
+      <c r="A12" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Clientes Inactivos</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Preparación de Material y Muestras</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
+      <c r="A13" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Clientes Nuevos / Potenciales</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Ruta del Día</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Competencia en la Zona</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Actividades Mes</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
+      <c r="A15" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Ventas por Cliente</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Plan de Acción</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A16" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Liquidación</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
+      <c r="A17" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Actividades de Impulso</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Despliegue y Revisión de Circulares</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Clientes Prioritarios</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Administración de Cartera</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
+      <c r="A19" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Estrategia por Producto</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Conciliación de Cartera</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
+      <c r="A20" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Metas de Venta del Mes</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Llamadas de Cobro</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Plan de Trabajo Diario</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Revisión de Cartera Vencida</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Confirmación de Citas</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Capacitación</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Preparación de Material y Muestras</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Interacción con Áreas</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
+      <c r="A24" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Programación de Visitas</t>
+          <t>Contabilidad y Cartera</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -3078,10 +3087,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
+      <c r="A25" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Ruta del Día</t>
+          <t>Dirección Técnica</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -3101,33 +3112,37 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Actividades Mes</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="A26" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Logística y Despachos</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
+      <c r="A27" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Activaciones en Punto de Venta</t>
+          <t>Mercadeo</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -3147,10 +3162,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
+      <c r="A28" s="11" t="n">
+        <v>5</v>
+      </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Capacitaciones a Clientes</t>
+          <t>RRHH</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -3170,55 +3187,55 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Eventos y Congresos</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Reunión Ventas</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Material POP</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Revisión Correos</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Administración de Cartera</t>
+          <t>Seguimientos</t>
         </is>
       </c>
       <c r="B31" s="6" t="n"/>
@@ -3232,761 +3249,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Acuerdos de Pago</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>Conciliación de Pagos</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>Llamadas de Cobro</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>Revisión de Cartera Vencida</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Capacitación</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>Herramientas (Epithelium Visita, Vademécum)</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="n"/>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Normatividad</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>Producto</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="11" t="n"/>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Técnicas de Venta</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Interacción con Áreas</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="11" t="n"/>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>Calidad</t>
-        </is>
-      </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="n"/>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Contabilidad y Cartera</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="11" t="n"/>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>Dirección Técnica</t>
-        </is>
-      </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D44" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="n"/>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>Logística y Despachos</t>
-        </is>
-      </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="11" t="n"/>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>Mercadeo</t>
-        </is>
-      </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D46" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="11" t="n"/>
-      <c r="B47" s="11" t="inlineStr">
-        <is>
-          <t>Producción</t>
-        </is>
-      </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Reunión Ventas</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="n"/>
-      <c r="B49" s="11" t="inlineStr">
-        <is>
-          <t>Comité Comercial</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D49" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="inlineStr">
-        <is>
-          <t>Reunión Semanal</t>
-        </is>
-      </c>
-      <c r="C50" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D50" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>Revisión de Resultados</t>
-        </is>
-      </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D51" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E51" s="12" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Revisión Correos</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="11" t="n"/>
-      <c r="B53" s="11" t="inlineStr">
-        <is>
-          <t>Comunicaciones Internas</t>
-        </is>
-      </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D53" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E53" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="11" t="inlineStr">
-        <is>
-          <t>Pedidos</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="11" t="inlineStr">
-        <is>
-          <t>Solicitudes de Clientes</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="11" t="n"/>
-      <c r="B57" s="11" t="inlineStr">
-        <is>
-          <t>Compromisos de Visita</t>
-        </is>
-      </c>
-      <c r="C57" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D57" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E57" s="12" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="11" t="n"/>
-      <c r="B58" s="11" t="inlineStr">
-        <is>
-          <t>Cotizaciones</t>
-        </is>
-      </c>
-      <c r="C58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="11" t="n"/>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>Muestras Entregadas</t>
-        </is>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="11" t="n"/>
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>Pedidos Pendientes</t>
-        </is>
-      </c>
-      <c r="C60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Trámites y Reclamos</t>
         </is>
       </c>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="11" t="n"/>
-      <c r="B62" s="11" t="inlineStr">
-        <is>
-          <t>Devoluciones</t>
-        </is>
-      </c>
-      <c r="C62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="11" t="n"/>
-      <c r="B63" s="11" t="inlineStr">
-        <is>
-          <t>Garantías</t>
-        </is>
-      </c>
-      <c r="C63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="11" t="n"/>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>Notas Crédito</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="n"/>
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>PQR de Clientes</t>
-        </is>
-      </c>
-      <c r="C65" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D65" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E65" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C5:E106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:E73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,✓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4077,60 +3367,60 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>X en los tipos de visita donde sale cada clasificación. Con X en Visita Médica y Visita Comercial (20 y 21) el vendedor marca una, otra o ambas; con las dos marcadas se usan los objetivos de "Visita Médica Comercial" (hoja Visitas).</t>
+          <t>X en los tipos de visita donde sale cada clasificación. Con X en Visita Médica y Visita Cliente (20 y 21) el vendedor marca una, otra o ambas; con las dos marcadas se usan los objetivos de "Visita Médica Comercial" (hoja Visitas).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Clasificación</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Clientes</t>
         </is>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Etiquetas en la maestra</t>
         </is>
       </c>
-      <c r="E4" s="25" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>Visita Médica</t>
         </is>
       </c>
-      <c r="F4" s="25" t="inlineStr">
-        <is>
-          <t>Visita Comercial</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Visita Cliente</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
         <is>
           <t>Punto de Venta</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="n">
+      <c r="A5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Tienda de piel pura con más de 3 puntos de venta</t>
         </is>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Cliente (5)</t>
         </is>
@@ -4144,18 +3434,18 @@
       <c r="G5" s="34" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Tienda de piel pura con 3 o menos puntos de venta</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Cliente (27)</t>
         </is>
@@ -4169,18 +3459,18 @@
       <c r="G6" s="34" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="n">
+      <c r="A7" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Punto de Venta Tienda Dermatologica</t>
         </is>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="19" t="n">
         <v>222</v>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Punto de Venta (220) · Centro de Distribucion (2)</t>
         </is>
@@ -4194,18 +3484,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="n">
+      <c r="A8" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Consultorio con razon social perteneciente a medico con venta al publico</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>Cliente (10)</t>
         </is>
@@ -4219,18 +3509,18 @@
       <c r="G8" s="34" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="n">
+      <c r="A9" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Centro médico o consultorio especializado en manejo de pies</t>
         </is>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Cliente (2)</t>
         </is>
@@ -4244,18 +3534,18 @@
       <c r="G9" s="34" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Socio Epithelium incluido en el panel</t>
         </is>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Medico Accionista - Panel Visita Medica (19) · Accionista Epithelium (2)</t>
         </is>
@@ -4273,18 +3563,18 @@
       <c r="G10" s="34" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="n">
+      <c r="A11" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="B11" s="26" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Médico compradores que no es socio y no tiene tienda de piel</t>
         </is>
       </c>
-      <c r="C11" s="25" t="n">
+      <c r="C11" s="19" t="n">
         <v>45</v>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Cliente - Medico Panel (42) · Cliente (2) · Medico Panel Visita Medica (1)</t>
         </is>
@@ -4302,18 +3592,18 @@
       <c r="G11" s="34" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="n">
+      <c r="A12" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Médico a visitar incluido en el panel</t>
         </is>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="C12" s="19" t="n">
         <v>207</v>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>Medico Panel Visita Medica (147) · Medico - Ateneo Sanitas - Centro Dermatologico Federico Lleras Acosta E.S.E (20) · Medico - Ateneo Hospital San Jose -Fundacion Universitaria de la Salud - FUCS (18) · Medico - Ateneo Universidad del Bosque (12) · Medico - Ateneo Hospital Militar Central (6) · Medico - Protocolo Medico (2) · Cliente - Medico Panel (2)</t>
         </is>
@@ -4327,18 +3617,18 @@
       <c r="G12" s="34" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n">
+      <c r="A13" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="B13" s="26" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Droguería con menos de 5 puntos de Venta</t>
         </is>
       </c>
-      <c r="C13" s="25" t="n">
+      <c r="C13" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="26" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Cliente (4)</t>
         </is>
@@ -4352,18 +3642,18 @@
       <c r="G13" s="34" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="n">
+      <c r="A14" s="19" t="n">
         <v>50</v>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Establecimientos comerciales tipo SPA donde se maneje la categoría</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Cliente (12)</t>
         </is>
@@ -4377,18 +3667,18 @@
       <c r="G14" s="34" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="n">
+      <c r="A15" s="19" t="n">
         <v>53</v>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Establecimientos comerciales de oportunidad donde se maneje la categoría. Eventos realizados, ferias, etc.</t>
         </is>
       </c>
-      <c r="C15" s="25" t="n">
+      <c r="C15" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="26" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Cliente (2)</t>
         </is>
@@ -4402,18 +3692,18 @@
       <c r="G15" s="34" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="n">
+      <c r="A16" s="19" t="n">
         <v>60</v>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>Asociaciones, clínicas, etc, cuyo capital es de origen privado</t>
         </is>
       </c>
-      <c r="C16" s="25" t="n">
+      <c r="C16" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="26" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>Cliente (3)</t>
         </is>
@@ -4427,18 +3717,18 @@
       <c r="G16" s="34" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="n">
+      <c r="A17" s="19" t="n">
         <v>61</v>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Entidades gubernamentales con citación a cotizar o licitación. No cuentan con precio fijo definido.</t>
         </is>
       </c>
-      <c r="C17" s="25" t="n">
+      <c r="C17" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="26" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>Cliente (1) · Entidad Gubernamental Cliente (1)</t>
         </is>
@@ -4452,18 +3742,18 @@
       <c r="G17" s="34" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="n">
+      <c r="A18" s="19" t="n">
         <v>70</v>
       </c>
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Cliente con bodega que hace distribución local. Maneja fuerza de ventas y visitadores.</t>
         </is>
       </c>
-      <c r="C18" s="25" t="n">
+      <c r="C18" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="26" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>Cliente (2)</t>
         </is>
@@ -4477,18 +3767,18 @@
       <c r="G18" s="34" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="n">
+      <c r="A19" s="19" t="n">
         <v>71</v>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>Cliente con bodega que hace distribución local. Maneja fuerza de ventas y visitadores en Bogotá y Área Metropolitana</t>
         </is>
       </c>
-      <c r="C19" s="25" t="n">
+      <c r="C19" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="26" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Cliente (4)</t>
         </is>
@@ -4502,18 +3792,18 @@
       <c r="G19" s="34" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="n">
+      <c r="A20" s="19" t="n">
         <v>90</v>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>Accionista Epithelium S.A. que tienen tienda de piel o punto de venta de facturacion al publico</t>
         </is>
       </c>
-      <c r="C20" s="25" t="n">
+      <c r="C20" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Cliente (10) · Accionista Epithelium (1)</t>
         </is>

</xml_diff>

<commit_message>
Contacto nuevo: teléfono obligatorio; Colocación con Presentación Portafolio y Creación Cliente para contactos nuevos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1455,64 +1455,42 @@
       <c r="I24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo Productos</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="n"/>
+      <c r="A25" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Presentación Portafolio</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Ajuste de Fórmula</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Creación Cliente</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
       <c r="F26" s="12" t="n"/>
       <c r="G26" s="12" t="inlineStr">
         <is>
@@ -1527,49 +1505,47 @@
       <c r="I26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Fórmula Magistral Nueva</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I27" s="12" t="n"/>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo Productos</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Muestra de Desarrollo</t>
+          <t>Ajuste de Fórmula</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1601,46 +1577,56 @@
       <c r="I28" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Devoluciones - PQR</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
+      <c r="A29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Fórmula Magistral Nueva</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Devolución</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="n"/>
+          <t>Muestra de Desarrollo</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1651,55 +1637,57 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I30" s="12" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>Queja</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="12" t="n"/>
-      <c r="I31" s="12" t="n"/>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Devoluciones - PQR</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Reacondicionamiento</t>
+          <t>Devolución</t>
         </is>
       </c>
       <c r="C32" s="12" t="n"/>
@@ -1713,18 +1701,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F32" s="12" t="n"/>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G32" s="12" t="n"/>
       <c r="H32" s="12" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Reclamo</t>
+          <t>Queja</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1753,18 +1745,14 @@
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Sugerencia</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Reacondicionamiento</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n"/>
       <c r="D34" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1775,65 +1763,51 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F34" s="12" t="n"/>
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Entrega de Muestras</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A35" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Reclamo</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
+      <c r="I35" s="12" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Muestra Comercial</t>
+          <t>Sugerencia</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -1856,66 +1830,72 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H36" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="12" t="n"/>
       <c r="I36" s="12" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>Muestra Médica</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="n"/>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I37" s="12" t="n"/>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Entrega de Muestras</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Tester</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
+          <t>Muestra Comercial</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1926,44 +1906,62 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="12" t="n"/>
-      <c r="I38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Exhibición</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
-      <c r="I39" s="7" t="n"/>
+      <c r="A39" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Muestra Médica</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Góndola</t>
+          <t>Tester</t>
         </is>
       </c>
       <c r="C40" s="12" t="n"/>
@@ -1980,40 +1978,42 @@
       </c>
       <c r="G40" s="12" t="n"/>
       <c r="H40" s="12" t="n"/>
-      <c r="I40" s="12" t="n"/>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>Material POP</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="n"/>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G41" s="12" t="n"/>
-      <c r="H41" s="12" t="n"/>
-      <c r="I41" s="12" t="n"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Exhibición</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n"/>
+      <c r="I41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Vitrina</t>
+          <t>Góndola</t>
         </is>
       </c>
       <c r="C42" s="12" t="n"/>
@@ -2033,89 +2033,89 @@
       <c r="I42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Mapa del Cliente</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="n"/>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n"/>
-      <c r="I43" s="7" t="n"/>
+      <c r="A43" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Material POP</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="12" t="n"/>
+      <c r="I43" s="12" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Portafolio Actual</t>
+          <t>Vitrina</t>
         </is>
       </c>
       <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="D44" s="12" t="n"/>
       <c r="E44" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F44" s="12" t="n"/>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G44" s="12" t="n"/>
       <c r="H44" s="12" t="n"/>
       <c r="I44" s="12" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>Productos Foco</t>
-        </is>
-      </c>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F45" s="12" t="n"/>
-      <c r="G45" s="12" t="n"/>
-      <c r="H45" s="12" t="n"/>
-      <c r="I45" s="12" t="n"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Mapa del Cliente</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="7" t="n"/>
+      <c r="I45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>Productos Nuevos</t>
+          <t>Portafolio Actual</t>
         </is>
       </c>
       <c r="C46" s="12" t="n"/>
@@ -2136,11 +2136,11 @@
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Productos Transición</t>
+          <t>Productos Foco</t>
         </is>
       </c>
       <c r="C47" s="12" t="n"/>
@@ -2160,65 +2160,73 @@
       <c r="I47" s="12" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>Parrilla Promocional</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="n"/>
-      <c r="H48" s="7" t="n"/>
-      <c r="I48" s="7" t="n"/>
+      <c r="A48" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Productos Nuevos</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n"/>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="12" t="n"/>
+      <c r="H48" s="12" t="n"/>
+      <c r="I48" s="12" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="n"/>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="n"/>
-      <c r="D49" s="10" t="n"/>
-      <c r="E49" s="10" t="n"/>
-      <c r="F49" s="10" t="n"/>
-      <c r="G49" s="10" t="n"/>
-      <c r="H49" s="10" t="n"/>
-      <c r="I49" s="10" t="n"/>
+      <c r="A49" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Productos Transición</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
+      <c r="I49" s="12" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Precios</t>
+          <t>Parrilla Promocional</t>
         </is>
       </c>
       <c r="B50" s="6" t="n"/>
-      <c r="C50" s="7" t="n"/>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="E50" s="7" t="n"/>
       <c r="F50" s="7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -2229,62 +2237,54 @@
       <c r="I50" s="7" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>Lista de Precios</t>
-        </is>
-      </c>
-      <c r="C51" s="12" t="n"/>
-      <c r="D51" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E51" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F51" s="12" t="n"/>
-      <c r="G51" s="12" t="n"/>
-      <c r="H51" s="12" t="n"/>
-      <c r="I51" s="12" t="n"/>
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="10" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="10" t="n"/>
+      <c r="I51" s="10" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>Negociación</t>
-        </is>
-      </c>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="n"/>
-      <c r="G52" s="12" t="n"/>
-      <c r="H52" s="12" t="n"/>
-      <c r="I52" s="12" t="n"/>
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Precios</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="n"/>
+      <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Chequeo de Precios</t>
+          <t>Lista de Precios</t>
         </is>
       </c>
       <c r="C53" s="12" t="n"/>
@@ -2298,72 +2298,46 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F53" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F53" s="12" t="n"/>
       <c r="G53" s="12" t="n"/>
       <c r="H53" s="12" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Productos Nuevos</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A54" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="n"/>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="n"/>
+      <c r="G54" s="12" t="n"/>
+      <c r="H54" s="12" t="n"/>
+      <c r="I54" s="12" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Codificación</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Chequeo de Precios</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n"/>
       <c r="D55" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -2374,51 +2348,65 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F55" s="12" t="n"/>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B56" s="11" t="inlineStr">
-        <is>
-          <t>Entrega de Muestra</t>
-        </is>
-      </c>
-      <c r="C56" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D56" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F56" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n"/>
-      <c r="I56" s="12" t="n"/>
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Productos Nuevos</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Material de Apoyo</t>
+          <t>Codificación</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
@@ -2436,22 +2424,18 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F57" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F57" s="12" t="n"/>
       <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Presentación del Producto</t>
+          <t>Entrega de Muestra</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
@@ -2474,56 +2458,50 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G58" s="12" t="n"/>
+      <c r="H58" s="12" t="n"/>
+      <c r="I58" s="12" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Protocolo Médico</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="n"/>
-      <c r="F59" s="7" t="n"/>
-      <c r="G59" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H59" s="7" t="n"/>
-      <c r="I59" s="7" t="n"/>
+      <c r="A59" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>Material de Apoyo</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E59" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G59" s="12" t="n"/>
+      <c r="H59" s="12" t="n"/>
+      <c r="I59" s="12" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Inscripción del Médico</t>
+          <t>Presentación del Producto</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
@@ -2536,48 +2514,66 @@
           <t>X</t>
         </is>
       </c>
-      <c r="E60" s="12" t="n"/>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="12" t="n"/>
-      <c r="H60" s="12" t="n"/>
-      <c r="I60" s="12" t="n"/>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B61" s="11" t="inlineStr">
-        <is>
-          <t>Presentación Protocolo Médico</t>
-        </is>
-      </c>
-      <c r="C61" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E61" s="12" t="n"/>
-      <c r="F61" s="12" t="n"/>
-      <c r="G61" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H61" s="12" t="n"/>
-      <c r="I61" s="12" t="n"/>
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Protocolo Médico</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n"/>
+      <c r="F61" s="7" t="n"/>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="n"/>
+      <c r="I61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Seguimiento</t>
+          <t>Inscripción del Médico</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
@@ -2598,11 +2594,11 @@
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Solicitud y Recolección de Información</t>
+          <t>Presentación Protocolo Médico</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
@@ -2617,9 +2613,63 @@
       </c>
       <c r="E63" s="12" t="n"/>
       <c r="F63" s="12" t="n"/>
-      <c r="G63" s="12" t="n"/>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Seguimiento</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="12" t="n"/>
+      <c r="I64" s="12" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>Solicitud y Recolección de Información</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="n"/>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+      <c r="I65" s="12" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Nombre de contacto en nombre propio y obligatorio; matriz nueva (categoría Lead para contactos nuevos); Lead visitado / no visitado en cian, también en el borde de la tarjeta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1310,16 +1310,8 @@
         </is>
       </c>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
       <c r="I20" s="7" t="n"/>
     </row>
     <row r="21">
@@ -1343,16 +1335,8 @@
         </is>
       </c>
       <c r="F21" s="12" t="n"/>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
       <c r="I21" s="12" t="n"/>
     </row>
     <row r="22">
@@ -1376,16 +1360,8 @@
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
       <c r="I22" s="12" t="n"/>
     </row>
     <row r="23">
@@ -1409,16 +1385,8 @@
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H23" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
       <c r="I23" s="12" t="n"/>
     </row>
     <row r="24">
@@ -1442,55 +1410,69 @@
         </is>
       </c>
       <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H24" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
       <c r="I24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Presentación Portafolio</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I25" s="12" t="n"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo Productos</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Creación Cliente</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
+          <t>Ajuste de Fórmula</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F26" s="12" t="n"/>
       <c r="G26" s="12" t="inlineStr">
         <is>
@@ -1505,47 +1487,49 @@
       <c r="I26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo Productos</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I27" s="7" t="n"/>
+      <c r="A27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Fórmula Magistral Nueva</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Ajuste de Fórmula</t>
+          <t>Muestra de Desarrollo</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1577,56 +1561,46 @@
       <c r="I28" s="12" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Fórmula Magistral Nueva</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H29" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="n"/>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Devoluciones - PQR</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Muestra de Desarrollo</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Devolución</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n"/>
       <c r="D30" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1637,57 +1611,55 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H30" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
       <c r="I30" s="12" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Devoluciones - PQR</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
+      <c r="A31" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Queja</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Devolución</t>
+          <t>Reacondicionamiento</t>
         </is>
       </c>
       <c r="C32" s="12" t="n"/>
@@ -1701,22 +1673,18 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F32" s="12" t="n"/>
       <c r="G32" s="12" t="n"/>
       <c r="H32" s="12" t="n"/>
       <c r="I32" s="12" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Queja</t>
+          <t>Reclamo</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1745,14 +1713,18 @@
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Reacondicionamiento</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="n"/>
+          <t>Sugerencia</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1763,51 +1735,65 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F34" s="12" t="n"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>Reclamo</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G35" s="12" t="n"/>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Entrega de Muestras</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Sugerencia</t>
+          <t>Muestra Comercial</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -1830,72 +1816,66 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="12" t="n"/>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I36" s="12" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Entrega de Muestras</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A37" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Muestra Médica</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Muestra Comercial</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
       <c r="E38" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -1906,62 +1886,44 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H38" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>Muestra Médica</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F39" s="12" t="n"/>
-      <c r="G39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H39" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I39" s="12" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Exhibición</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Tester</t>
+          <t>Góndola</t>
         </is>
       </c>
       <c r="C40" s="12" t="n"/>
@@ -1978,42 +1940,40 @@
       </c>
       <c r="G40" s="12" t="n"/>
       <c r="H40" s="12" t="n"/>
-      <c r="I40" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I40" s="12" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Exhibición</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n"/>
-      <c r="I41" s="7" t="n"/>
+      <c r="A41" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Material POP</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n"/>
+      <c r="D41" s="12" t="n"/>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41" s="12" t="n"/>
+      <c r="I41" s="12" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Góndola</t>
+          <t>Vitrina</t>
         </is>
       </c>
       <c r="C42" s="12" t="n"/>
@@ -2033,89 +1993,89 @@
       <c r="I42" s="12" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Material POP</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G43" s="12" t="n"/>
-      <c r="H43" s="12" t="n"/>
-      <c r="I43" s="12" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Mapa del Cliente</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Vitrina</t>
+          <t>Portafolio Actual</t>
         </is>
       </c>
       <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="F44" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F44" s="12" t="n"/>
       <c r="G44" s="12" t="n"/>
       <c r="H44" s="12" t="n"/>
       <c r="I44" s="12" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Mapa del Cliente</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
+      <c r="A45" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Productos Foco</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="12" t="n"/>
+      <c r="I45" s="12" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>Portafolio Actual</t>
+          <t>Productos Nuevos</t>
         </is>
       </c>
       <c r="C46" s="12" t="n"/>
@@ -2136,11 +2096,11 @@
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Productos Foco</t>
+          <t>Productos Transición</t>
         </is>
       </c>
       <c r="C47" s="12" t="n"/>
@@ -2160,73 +2120,65 @@
       <c r="I47" s="12" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B48" s="11" t="inlineStr">
-        <is>
-          <t>Productos Nuevos</t>
-        </is>
-      </c>
-      <c r="C48" s="12" t="n"/>
-      <c r="D48" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="12" t="n"/>
-      <c r="H48" s="12" t="n"/>
-      <c r="I48" s="12" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Parrilla Promocional</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
+      <c r="I48" s="7" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B49" s="11" t="inlineStr">
-        <is>
-          <t>Productos Transición</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="n"/>
-      <c r="D49" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="12" t="n"/>
-      <c r="H49" s="12" t="n"/>
-      <c r="I49" s="12" t="n"/>
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="n"/>
+      <c r="D49" s="10" t="n"/>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="10" t="n"/>
+      <c r="I49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Parrilla Promocional</t>
+          <t>Precios</t>
         </is>
       </c>
       <c r="B50" s="6" t="n"/>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C50" s="7" t="n"/>
       <c r="D50" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="E50" s="7" t="n"/>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -2237,54 +2189,62 @@
       <c r="I50" s="7" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="n"/>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="C51" s="10" t="n"/>
-      <c r="D51" s="10" t="n"/>
-      <c r="E51" s="10" t="n"/>
-      <c r="F51" s="10" t="n"/>
-      <c r="G51" s="10" t="n"/>
-      <c r="H51" s="10" t="n"/>
-      <c r="I51" s="10" t="n"/>
+      <c r="A51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Lista de Precios</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="12" t="n"/>
+      <c r="I51" s="12" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Precios</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="n"/>
-      <c r="H52" s="7" t="n"/>
-      <c r="I52" s="7" t="n"/>
+      <c r="A52" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
+      <c r="I52" s="12" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>Lista de Precios</t>
+          <t>Chequeo de Precios</t>
         </is>
       </c>
       <c r="C53" s="12" t="n"/>
@@ -2298,46 +2258,60 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F53" s="12" t="n"/>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G53" s="12" t="n"/>
       <c r="H53" s="12" t="n"/>
       <c r="I53" s="12" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B54" s="11" t="inlineStr">
-        <is>
-          <t>Negociación</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="n"/>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F54" s="12" t="n"/>
-      <c r="G54" s="12" t="n"/>
-      <c r="H54" s="12" t="n"/>
-      <c r="I54" s="12" t="n"/>
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Productos Nuevos</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="n"/>
+      <c r="H54" s="7" t="n"/>
+      <c r="I54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Chequeo de Precios</t>
-        </is>
-      </c>
-      <c r="C55" s="12" t="n"/>
+          <t>Codificación</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D55" s="12" t="inlineStr">
         <is>
           <t>X</t>
@@ -2348,65 +2322,51 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="F55" s="12" t="n"/>
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Productos Nuevos</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="A56" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Entrega de Muestra</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G56" s="12" t="n"/>
+      <c r="H56" s="12" t="n"/>
+      <c r="I56" s="12" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Codificación</t>
+          <t>Material de Apoyo</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
@@ -2424,18 +2384,22 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F57" s="12" t="n"/>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="12" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Entrega de Muestra</t>
+          <t>Presentación del Producto</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
@@ -2463,117 +2427,85 @@
       <c r="I58" s="12" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>Material de Apoyo</t>
-        </is>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F59" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G59" s="12" t="n"/>
-      <c r="H59" s="12" t="n"/>
-      <c r="I59" s="12" t="n"/>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Protocolo Médico</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="7" t="n"/>
+      <c r="H59" s="7" t="n"/>
+      <c r="I59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Inscripción del Médico</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="12" t="n"/>
+      <c r="I60" s="12" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>Presentación del Producto</t>
-        </is>
-      </c>
-      <c r="C60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="F60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>Protocolo Médico</t>
-        </is>
-      </c>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="n"/>
-      <c r="F61" s="7" t="n"/>
-      <c r="G61" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H61" s="7" t="n"/>
-      <c r="I61" s="7" t="n"/>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Presentación Protocolo Médico</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
+      <c r="H61" s="12" t="n"/>
+      <c r="I61" s="12" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Inscripción del Médico</t>
+          <t>Seguimiento</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
@@ -2594,11 +2526,11 @@
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Presentación Protocolo Médico</t>
+          <t>Solicitud y Recolección de Información</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
@@ -2613,67 +2545,235 @@
       </c>
       <c r="E63" s="12" t="n"/>
       <c r="F63" s="12" t="n"/>
-      <c r="G63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G63" s="12" t="n"/>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>Seguimiento</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="12" t="n"/>
-      <c r="I64" s="12" t="n"/>
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="7" t="n"/>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="7" t="n"/>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Solicitud y Recolección de Información</t>
-        </is>
-      </c>
-      <c r="C65" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="D65" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>Presentación Compañía</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
       <c r="E65" s="12" t="n"/>
       <c r="F65" s="12" t="n"/>
-      <c r="G65" s="12" t="n"/>
-      <c r="H65" s="12" t="n"/>
-      <c r="I65" s="12" t="n"/>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I65" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Presentación Portafolio</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="12" t="n"/>
+      <c r="E66" s="12" t="n"/>
+      <c r="F66" s="12" t="n"/>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I66" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>Condiciones Comerciales</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H67" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I67" s="12" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>Actividades</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H68" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I68" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="C69" s="12" t="n"/>
+      <c r="D69" s="12" t="n"/>
+      <c r="E69" s="12" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H69" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>Solicitud de Creación</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="n"/>
+      <c r="D70" s="12" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H70" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>Protocolo Médico</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="n"/>
+      <c r="D71" s="12" t="n"/>
+      <c r="E71" s="12" t="n"/>
+      <c r="F71" s="12" t="n"/>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I71" s="12" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C5:I104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:I106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,✓"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Matriz: se quita Mapa del Cliente de Visita Médica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Índice" sheetId="1" state="visible" r:id="rId1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Actualizada el 01/10/2026 · es lo que la app tiene cargado hoy</t>
+          <t>Actualizada el 02/10/2026 · es lo que la app tiene cargado hoy</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1999,11 +1999,7 @@
         </is>
       </c>
       <c r="B43" s="6" t="n"/>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C43" s="7" t="n"/>
       <c r="D43" s="7" t="inlineStr">
         <is>
           <t>✓</t>
@@ -2788,7 +2784,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -2809,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44.1" customHeight="1">
+    <row r="4" ht="44.15" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Categoría</t>
@@ -3441,7 +3437,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Mercadeo: trabajo administrativo de la Coordinadora Comercial con texto por objetivo y proyectos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Objetivos y subcategorías de Oficina, Fuera de la Oficina y Planeación Mes.</t>
+          <t>Objetivos y subcategorías de Oficina, Fuera de la Oficina, Planeación Mes y Mercadeo (solo Coordinadora Comercial).</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2783,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -2831,6 +2833,11 @@
           <t>Planeación Mes</t>
         </is>
       </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Mercadeo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2846,6 +2853,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
@@ -2863,6 +2871,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F6" s="12" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
@@ -2880,6 +2889,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F7" s="12" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2895,6 +2905,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2910,6 +2921,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2929,6 +2941,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
@@ -2950,6 +2963,7 @@
         </is>
       </c>
       <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">
@@ -2971,6 +2985,7 @@
         </is>
       </c>
       <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n">
@@ -2992,6 +3007,7 @@
         </is>
       </c>
       <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -3015,6 +3031,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n">
@@ -3036,6 +3053,7 @@
         </is>
       </c>
       <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n">
@@ -3057,6 +3075,7 @@
         </is>
       </c>
       <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">
@@ -3078,6 +3097,7 @@
         </is>
       </c>
       <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3097,6 +3117,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
@@ -3118,6 +3139,7 @@
         </is>
       </c>
       <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">
@@ -3139,6 +3161,7 @@
         </is>
       </c>
       <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -3160,6 +3183,7 @@
         </is>
       </c>
       <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -3183,6 +3207,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -3206,6 +3231,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
@@ -3231,6 +3257,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F24" s="12" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
@@ -3256,6 +3283,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F25" s="12" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -3281,6 +3309,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F26" s="12" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -3306,6 +3335,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F27" s="12" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -3331,6 +3361,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="F28" s="12" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -3354,6 +3385,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -3377,6 +3409,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3396,6 +3429,7 @@
         </is>
       </c>
       <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3415,6 +3449,71 @@
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Proyectos</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo Actividades Comerciales</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Investigación de Mercado</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Contacto Proveedores</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
Mercadeo: Contacto Cliente y Contacto Proveedores dentro de Proyectos; nueva Visita Ateneo Médico abierta a todas las zonas; script del módulo de pruebas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Actualizada el 02/10/2026 · es lo que la app tiene cargado hoy</t>
+          <t>Actualizada el 03/10/2026 · es lo que la app tiene cargado hoy</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -852,6 +852,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -921,6 +922,11 @@
           <t>Contacto nuevo · Punto de Venta</t>
         </is>
       </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Visita Ateneo Médico</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -952,6 +958,11 @@
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
@@ -967,6 +978,7 @@
       <c r="G6" s="10" t="n"/>
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -990,6 +1002,7 @@
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
@@ -1015,6 +1028,7 @@
       <c r="G8" s="12" t="n"/>
       <c r="H8" s="12" t="n"/>
       <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
@@ -1040,6 +1054,7 @@
       <c r="G9" s="12" t="n"/>
       <c r="H9" s="12" t="n"/>
       <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
@@ -1065,6 +1080,7 @@
       <c r="G10" s="12" t="n"/>
       <c r="H10" s="12" t="n"/>
       <c r="I10" s="12" t="n"/>
+      <c r="J10" s="12" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
@@ -1090,6 +1106,7 @@
       <c r="G11" s="12" t="n"/>
       <c r="H11" s="12" t="n"/>
       <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1113,6 +1130,7 @@
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n">
@@ -1138,6 +1156,7 @@
       <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="n"/>
       <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n">
@@ -1163,6 +1182,7 @@
       <c r="G14" s="12" t="n"/>
       <c r="H14" s="12" t="n"/>
       <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n">
@@ -1188,6 +1208,7 @@
       <c r="G15" s="12" t="n"/>
       <c r="H15" s="12" t="n"/>
       <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1215,6 +1236,7 @@
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">
@@ -1240,6 +1262,7 @@
       <c r="G17" s="12" t="n"/>
       <c r="H17" s="12" t="n"/>
       <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n">
@@ -1269,6 +1292,7 @@
       <c r="G18" s="12" t="n"/>
       <c r="H18" s="12" t="n"/>
       <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
@@ -1290,6 +1314,7 @@
       <c r="G19" s="12" t="n"/>
       <c r="H19" s="12" t="n"/>
       <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1313,6 +1338,7 @@
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n"/>
       <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1338,6 +1364,7 @@
       <c r="G21" s="12" t="n"/>
       <c r="H21" s="12" t="n"/>
       <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1363,6 +1390,7 @@
       <c r="G22" s="12" t="n"/>
       <c r="H22" s="12" t="n"/>
       <c r="I22" s="12" t="n"/>
+      <c r="J22" s="12" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1388,6 +1416,7 @@
       <c r="G23" s="12" t="n"/>
       <c r="H23" s="12" t="n"/>
       <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
@@ -1413,6 +1442,7 @@
       <c r="G24" s="12" t="n"/>
       <c r="H24" s="12" t="n"/>
       <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1448,6 +1478,11 @@
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1485,6 +1520,11 @@
         </is>
       </c>
       <c r="I26" s="12" t="n"/>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1522,6 +1562,11 @@
         </is>
       </c>
       <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1559,6 +1604,11 @@
         </is>
       </c>
       <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1590,6 +1640,11 @@
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1619,6 +1674,7 @@
       <c r="G30" s="12" t="n"/>
       <c r="H30" s="12" t="n"/>
       <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1652,6 +1708,11 @@
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="12" t="n"/>
       <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1677,6 +1738,7 @@
       <c r="G32" s="12" t="n"/>
       <c r="H32" s="12" t="n"/>
       <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
@@ -1710,6 +1772,11 @@
       <c r="G33" s="12" t="n"/>
       <c r="H33" s="12" t="n"/>
       <c r="I33" s="12" t="n"/>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1743,6 +1810,11 @@
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1782,6 +1854,11 @@
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
@@ -1827,6 +1904,11 @@
         </is>
       </c>
       <c r="I36" s="12" t="n"/>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1864,6 +1946,11 @@
         </is>
       </c>
       <c r="I37" s="12" t="n"/>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -1893,6 +1980,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J38" s="12" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -1916,6 +2004,7 @@
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
+      <c r="J39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
@@ -1941,6 +2030,7 @@
       <c r="G40" s="12" t="n"/>
       <c r="H40" s="12" t="n"/>
       <c r="I40" s="12" t="n"/>
+      <c r="J40" s="12" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
@@ -1966,6 +2056,7 @@
       <c r="G41" s="12" t="n"/>
       <c r="H41" s="12" t="n"/>
       <c r="I41" s="12" t="n"/>
+      <c r="J41" s="12" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
@@ -1991,6 +2082,7 @@
       <c r="G42" s="12" t="n"/>
       <c r="H42" s="12" t="n"/>
       <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2014,6 +2106,7 @@
       <c r="G43" s="7" t="n"/>
       <c r="H43" s="7" t="n"/>
       <c r="I43" s="7" t="n"/>
+      <c r="J43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
@@ -2039,6 +2132,7 @@
       <c r="G44" s="12" t="n"/>
       <c r="H44" s="12" t="n"/>
       <c r="I44" s="12" t="n"/>
+      <c r="J44" s="12" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n">
@@ -2064,6 +2158,7 @@
       <c r="G45" s="12" t="n"/>
       <c r="H45" s="12" t="n"/>
       <c r="I45" s="12" t="n"/>
+      <c r="J45" s="12" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
@@ -2089,6 +2184,7 @@
       <c r="G46" s="12" t="n"/>
       <c r="H46" s="12" t="n"/>
       <c r="I46" s="12" t="n"/>
+      <c r="J46" s="12" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
@@ -2114,6 +2210,7 @@
       <c r="G47" s="12" t="n"/>
       <c r="H47" s="12" t="n"/>
       <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -2141,6 +2238,11 @@
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
       <c r="I48" s="7" t="n"/>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -2156,6 +2258,7 @@
       <c r="G49" s="10" t="n"/>
       <c r="H49" s="10" t="n"/>
       <c r="I49" s="10" t="n"/>
+      <c r="J49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -2183,6 +2286,7 @@
       <c r="G50" s="7" t="n"/>
       <c r="H50" s="7" t="n"/>
       <c r="I50" s="7" t="n"/>
+      <c r="J50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
@@ -2208,6 +2312,7 @@
       <c r="G51" s="12" t="n"/>
       <c r="H51" s="12" t="n"/>
       <c r="I51" s="12" t="n"/>
+      <c r="J51" s="12" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
@@ -2233,6 +2338,7 @@
       <c r="G52" s="12" t="n"/>
       <c r="H52" s="12" t="n"/>
       <c r="I52" s="12" t="n"/>
+      <c r="J52" s="12" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
@@ -2262,6 +2368,7 @@
       <c r="G53" s="12" t="n"/>
       <c r="H53" s="12" t="n"/>
       <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -2293,6 +2400,11 @@
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="7" t="n"/>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
@@ -2322,6 +2434,11 @@
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2355,6 +2472,11 @@
       <c r="G56" s="12" t="n"/>
       <c r="H56" s="12" t="n"/>
       <c r="I56" s="12" t="n"/>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -2388,6 +2510,11 @@
       <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="12" t="n"/>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -2421,6 +2548,11 @@
       <c r="G58" s="12" t="n"/>
       <c r="H58" s="12" t="n"/>
       <c r="I58" s="12" t="n"/>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -2444,6 +2576,11 @@
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2469,6 +2606,11 @@
       <c r="G60" s="12" t="n"/>
       <c r="H60" s="12" t="n"/>
       <c r="I60" s="12" t="n"/>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -2494,6 +2636,11 @@
       <c r="G61" s="12" t="n"/>
       <c r="H61" s="12" t="n"/>
       <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -2519,6 +2666,11 @@
       <c r="G62" s="12" t="n"/>
       <c r="H62" s="12" t="n"/>
       <c r="I62" s="12" t="n"/>
+      <c r="J62" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -2544,6 +2696,11 @@
       <c r="G63" s="12" t="n"/>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
+      <c r="J63" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2571,6 +2728,7 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="J64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
@@ -2600,6 +2758,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J65" s="12" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n">
@@ -2629,6 +2788,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J66" s="12" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n">
@@ -2654,6 +2814,7 @@
         </is>
       </c>
       <c r="I67" s="12" t="n"/>
+      <c r="J67" s="12" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n">
@@ -2683,6 +2844,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J68" s="12" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n">
@@ -2712,6 +2874,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J69" s="12" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n">
@@ -2741,6 +2904,7 @@
           <t>X</t>
         </is>
       </c>
+      <c r="J70" s="12" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n">
@@ -2766,6 +2930,7 @@
         </is>
       </c>
       <c r="I71" s="12" t="n"/>
+      <c r="J71" s="12" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2783,7 +2948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3472,41 +3637,45 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo Actividades Comerciales</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="A34" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Contacto Cliente</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Investigación de Mercado</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="A35" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Contacto Proveedores</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Contacto Proveedores</t>
+          <t>Desarrollo Actividades Comerciales</t>
         </is>
       </c>
       <c r="B36" s="6" t="n"/>
@@ -3514,6 +3683,22 @@
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Investigación de Mercado</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
Visita Ateneo Médico: solo clasificación 61 y objetivos de Mercadeo con texto por objetivo y proyectos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -958,11 +958,7 @@
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
@@ -1478,11 +1474,7 @@
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1520,11 +1512,7 @@
         </is>
       </c>
       <c r="I26" s="12" t="n"/>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J26" s="12" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1562,11 +1550,7 @@
         </is>
       </c>
       <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J27" s="12" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1604,11 +1588,7 @@
         </is>
       </c>
       <c r="I28" s="12" t="n"/>
-      <c r="J28" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J28" s="12" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1640,11 +1620,7 @@
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1708,11 +1684,7 @@
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="12" t="n"/>
       <c r="I31" s="12" t="n"/>
-      <c r="J31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J31" s="12" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1772,11 +1744,7 @@
       <c r="G33" s="12" t="n"/>
       <c r="H33" s="12" t="n"/>
       <c r="I33" s="12" t="n"/>
-      <c r="J33" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J33" s="12" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1810,11 +1778,7 @@
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J34" s="12" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1858,11 +1822,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1904,11 +1864,7 @@
         </is>
       </c>
       <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J36" s="12" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1946,11 +1902,7 @@
         </is>
       </c>
       <c r="I37" s="12" t="n"/>
-      <c r="J37" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J37" s="12" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -2238,11 +2190,7 @@
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
       <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -2400,11 +2348,7 @@
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="7" t="n"/>
-      <c r="J54" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
@@ -2434,11 +2378,7 @@
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J55" s="12" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2472,11 +2412,7 @@
       <c r="G56" s="12" t="n"/>
       <c r="H56" s="12" t="n"/>
       <c r="I56" s="12" t="n"/>
-      <c r="J56" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J56" s="12" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -2510,11 +2446,7 @@
       <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="12" t="n"/>
-      <c r="J57" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J57" s="12" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -2548,11 +2480,7 @@
       <c r="G58" s="12" t="n"/>
       <c r="H58" s="12" t="n"/>
       <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J58" s="12" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -2576,11 +2504,7 @@
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
-      <c r="J59" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2606,11 +2530,7 @@
       <c r="G60" s="12" t="n"/>
       <c r="H60" s="12" t="n"/>
       <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -2636,11 +2556,7 @@
       <c r="G61" s="12" t="n"/>
       <c r="H61" s="12" t="n"/>
       <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J61" s="12" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -2666,11 +2582,7 @@
       <c r="G62" s="12" t="n"/>
       <c r="H62" s="12" t="n"/>
       <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -2696,11 +2608,7 @@
       <c r="G63" s="12" t="n"/>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J63" s="12" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2931,6 +2839,110 @@
       </c>
       <c r="I71" s="12" t="n"/>
       <c r="J71" s="12" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Proyectos</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="7" t="n"/>
+      <c r="D72" s="7" t="n"/>
+      <c r="E72" s="7" t="n"/>
+      <c r="F72" s="7" t="n"/>
+      <c r="G72" s="7" t="n"/>
+      <c r="H72" s="7" t="n"/>
+      <c r="I72" s="7" t="n"/>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>Contacto Cliente</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="n"/>
+      <c r="D73" s="10" t="n"/>
+      <c r="E73" s="10" t="n"/>
+      <c r="F73" s="10" t="n"/>
+      <c r="G73" s="10" t="n"/>
+      <c r="H73" s="10" t="n"/>
+      <c r="I73" s="10" t="n"/>
+      <c r="J73" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>Contacto Proveedores</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="10" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="10" t="n"/>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="10" t="n"/>
+      <c r="J74" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo Actividades Comerciales</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="7" t="n"/>
+      <c r="E75" s="7" t="n"/>
+      <c r="F75" s="7" t="n"/>
+      <c r="G75" s="7" t="n"/>
+      <c r="H75" s="7" t="n"/>
+      <c r="I75" s="7" t="n"/>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Investigación de Mercado</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="7" t="n"/>
+      <c r="F76" s="7" t="n"/>
+      <c r="G76" s="7" t="n"/>
+      <c r="H76" s="7" t="n"/>
+      <c r="I76" s="7" t="n"/>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Visita Ateneo Médico vuelve a los objetivos de Visita Médica; los objetivos con texto quedan solo en Mercadeo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -958,7 +958,11 @@
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
@@ -1474,7 +1478,11 @@
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="n"/>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1512,7 +1520,11 @@
         </is>
       </c>
       <c r="I26" s="12" t="n"/>
-      <c r="J26" s="12" t="n"/>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1550,7 +1562,11 @@
         </is>
       </c>
       <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="n"/>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1588,7 +1604,11 @@
         </is>
       </c>
       <c r="I28" s="12" t="n"/>
-      <c r="J28" s="12" t="n"/>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1620,7 +1640,11 @@
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1684,7 +1708,11 @@
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="12" t="n"/>
       <c r="I31" s="12" t="n"/>
-      <c r="J31" s="12" t="n"/>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1744,7 +1772,11 @@
       <c r="G33" s="12" t="n"/>
       <c r="H33" s="12" t="n"/>
       <c r="I33" s="12" t="n"/>
-      <c r="J33" s="12" t="n"/>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1778,7 +1810,11 @@
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="n"/>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1822,7 +1858,11 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="J35" s="7" t="n"/>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -1864,7 +1904,11 @@
         </is>
       </c>
       <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="n"/>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -1902,7 +1946,11 @@
         </is>
       </c>
       <c r="I37" s="12" t="n"/>
-      <c r="J37" s="12" t="n"/>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -2190,7 +2238,11 @@
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
       <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="n"/>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -2348,7 +2400,11 @@
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="7" t="n"/>
-      <c r="J54" s="7" t="n"/>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
@@ -2378,7 +2434,11 @@
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="n"/>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2412,7 +2472,11 @@
       <c r="G56" s="12" t="n"/>
       <c r="H56" s="12" t="n"/>
       <c r="I56" s="12" t="n"/>
-      <c r="J56" s="12" t="n"/>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -2446,7 +2510,11 @@
       <c r="G57" s="12" t="n"/>
       <c r="H57" s="12" t="n"/>
       <c r="I57" s="12" t="n"/>
-      <c r="J57" s="12" t="n"/>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -2480,7 +2548,11 @@
       <c r="G58" s="12" t="n"/>
       <c r="H58" s="12" t="n"/>
       <c r="I58" s="12" t="n"/>
-      <c r="J58" s="12" t="n"/>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -2504,7 +2576,11 @@
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
-      <c r="J59" s="7" t="n"/>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2530,7 +2606,11 @@
       <c r="G60" s="12" t="n"/>
       <c r="H60" s="12" t="n"/>
       <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="n"/>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -2556,7 +2636,11 @@
       <c r="G61" s="12" t="n"/>
       <c r="H61" s="12" t="n"/>
       <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="n"/>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -2582,7 +2666,11 @@
       <c r="G62" s="12" t="n"/>
       <c r="H62" s="12" t="n"/>
       <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="n"/>
+      <c r="J62" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -2608,7 +2696,11 @@
       <c r="G63" s="12" t="n"/>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="n"/>
+      <c r="J63" s="12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2839,110 +2931,6 @@
       </c>
       <c r="I71" s="12" t="n"/>
       <c r="J71" s="12" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>Proyectos</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="n"/>
-      <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="n"/>
-      <c r="E72" s="7" t="n"/>
-      <c r="F72" s="7" t="n"/>
-      <c r="G72" s="7" t="n"/>
-      <c r="H72" s="7" t="n"/>
-      <c r="I72" s="7" t="n"/>
-      <c r="J72" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B73" s="9" t="inlineStr">
-        <is>
-          <t>Contacto Cliente</t>
-        </is>
-      </c>
-      <c r="C73" s="10" t="n"/>
-      <c r="D73" s="10" t="n"/>
-      <c r="E73" s="10" t="n"/>
-      <c r="F73" s="10" t="n"/>
-      <c r="G73" s="10" t="n"/>
-      <c r="H73" s="10" t="n"/>
-      <c r="I73" s="10" t="n"/>
-      <c r="J73" s="10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B74" s="9" t="inlineStr">
-        <is>
-          <t>Contacto Proveedores</t>
-        </is>
-      </c>
-      <c r="C74" s="10" t="n"/>
-      <c r="D74" s="10" t="n"/>
-      <c r="E74" s="10" t="n"/>
-      <c r="F74" s="10" t="n"/>
-      <c r="G74" s="10" t="n"/>
-      <c r="H74" s="10" t="n"/>
-      <c r="I74" s="10" t="n"/>
-      <c r="J74" s="10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>Desarrollo Actividades Comerciales</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="n"/>
-      <c r="C75" s="7" t="n"/>
-      <c r="D75" s="7" t="n"/>
-      <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="n"/>
-      <c r="G75" s="7" t="n"/>
-      <c r="H75" s="7" t="n"/>
-      <c r="I75" s="7" t="n"/>
-      <c r="J75" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="5" t="inlineStr">
-        <is>
-          <t>Investigación de Mercado</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="n"/>
-      <c r="E76" s="7" t="n"/>
-      <c r="F76" s="7" t="n"/>
-      <c r="G76" s="7" t="n"/>
-      <c r="H76" s="7" t="n"/>
-      <c r="I76" s="7" t="n"/>
-      <c r="J76" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Visita Ateneo Médico: sin Desarrollo Productos, Devoluciones - PQR ni Protocolo Médico; Productos Nuevos sin Codificación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Matriz_App.xlsx
+++ b/datos/Matriz_App.xlsx
@@ -1478,11 +1478,7 @@
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1520,11 +1516,7 @@
         </is>
       </c>
       <c r="I26" s="12" t="n"/>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J26" s="12" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1562,11 +1554,7 @@
         </is>
       </c>
       <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J27" s="12" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1604,11 +1592,7 @@
         </is>
       </c>
       <c r="I28" s="12" t="n"/>
-      <c r="J28" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J28" s="12" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1640,11 +1624,7 @@
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1708,11 +1688,7 @@
       <c r="G31" s="12" t="n"/>
       <c r="H31" s="12" t="n"/>
       <c r="I31" s="12" t="n"/>
-      <c r="J31" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J31" s="12" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -1772,11 +1748,7 @@
       <c r="G33" s="12" t="n"/>
       <c r="H33" s="12" t="n"/>
       <c r="I33" s="12" t="n"/>
-      <c r="J33" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J33" s="12" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -1810,11 +1782,7 @@
       <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J34" s="12" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2434,11 +2402,7 @@
       <c r="G55" s="12" t="n"/>
       <c r="H55" s="12" t="n"/>
       <c r="I55" s="12" t="n"/>
-      <c r="J55" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J55" s="12" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2576,11 +2540,7 @@
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
-      <c r="J59" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="J59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2606,11 +2566,7 @@
       <c r="G60" s="12" t="n"/>
       <c r="H60" s="12" t="n"/>
       <c r="I60" s="12" t="n"/>
-      <c r="J60" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -2636,11 +2592,7 @@
       <c r="G61" s="12" t="n"/>
       <c r="H61" s="12" t="n"/>
       <c r="I61" s="12" t="n"/>
-      <c r="J61" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J61" s="12" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -2666,11 +2618,7 @@
       <c r="G62" s="12" t="n"/>
       <c r="H62" s="12" t="n"/>
       <c r="I62" s="12" t="n"/>
-      <c r="J62" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -2696,11 +2644,7 @@
       <c r="G63" s="12" t="n"/>
       <c r="H63" s="12" t="n"/>
       <c r="I63" s="12" t="n"/>
-      <c r="J63" s="12" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J63" s="12" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">

</xml_diff>